<commit_message>
Correct answer not working, test
</commit_message>
<xml_diff>
--- a/Questions - Round 1.xlsx
+++ b/Questions - Round 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cafnzholding-my.sharepoint.com/personal/thom_van_dusschoten_synerlogic_nl/Documents/Documenten/GitHub/Sustainability-quiz-TEST/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="130" documentId="11_DC4634EEB09B7631DD1D459FDEF3484CE4F5FC66" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A0C93D3-8B28-4AC3-A0F9-C26694C97848}"/>
+  <xr:revisionPtr revIDLastSave="134" documentId="11_DC4634EEB09B7631DD1D459FDEF3484CE4F5FC66" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64D53E76-6D31-4E43-825B-9B71E914DE4E}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EN" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="113">
   <si>
     <t>type</t>
   </si>
@@ -77,48 +77,9 @@
     <t>single</t>
   </si>
   <si>
-    <t>What is the main idea behind SDG 3 – Good Health and Well-Being?</t>
-  </si>
-  <si>
-    <t>Easy · Single choice</t>
-  </si>
-  <si>
-    <t>It focuses on workplace health and safety.</t>
-  </si>
-  <si>
-    <t>It only applies to national governments.</t>
-  </si>
-  <si>
-    <t>It asks companies to ignore long-term impacts.</t>
-  </si>
-  <si>
-    <t>It is only a marketing slogan with no practical meaning.</t>
-  </si>
-  <si>
-    <t>SDG 3 is about workplace health and safety and turning that goal into practical action. SDG 3 becomes useful when people translate the broad goal into practical decisions.</t>
-  </si>
-  <si>
     <t>Okay</t>
   </si>
   <si>
-    <t>What is STOCKMEIER’s stated ambition related to safety?</t>
-  </si>
-  <si>
-    <t>Replacing all safety training with posters</t>
-  </si>
-  <si>
-    <t>Zero work-related accidents</t>
-  </si>
-  <si>
-    <t>Only reducing accidents in offices</t>
-  </si>
-  <si>
-    <t>Accepting accidents if production targets are met</t>
-  </si>
-  <si>
-    <t>The report states an ambition for zero work-related accidents and zero harmful effects on health. STOCKMEIER examples make the SDG concrete and show how Group initiatives connect to global goals.</t>
-  </si>
-  <si>
     <t>Wat is het belangrijkste idee achter SDG 3 – Goede gezondheid en welzijn?</t>
   </si>
   <si>
@@ -161,45 +122,6 @@
     <t>Het rapport vermeldt de ambitie van nul werkgerelateerde ongevallen en nul schadelijke gevolgen voor de gezondheid. Voorbeelden van STOCKMEIER maken de SDG concreet en tonen hoe initiatieven van de Groep aansluiten bij wereldwijde doelen.</t>
   </si>
   <si>
-    <t>Was ist die zentrale Idee hinter SDG 3 – Gesundheit und Wohlergehen?</t>
-  </si>
-  <si>
-    <t>Leicht · Einfachauswahl</t>
-  </si>
-  <si>
-    <t>Es konzentriert sich auf Gesundheit und Sicherheit am Arbeitsplatz.</t>
-  </si>
-  <si>
-    <t>Es gilt nur für nationale Regierungen.</t>
-  </si>
-  <si>
-    <t>Es fordert Unternehmen auf, langfristige Auswirkungen zu ignorieren.</t>
-  </si>
-  <si>
-    <t>Es ist nur ein Marketingslogan ohne praktische Bedeutung.</t>
-  </si>
-  <si>
-    <t>Bei SDG 3 geht es um Gesundheit und Sicherheit am Arbeitsplatz und darum, dieses Ziel in konkrete Maßnahmen umzusetzen. SDG 3 wird nützlich, wenn Menschen das übergeordnete Ziel in praktische Entscheidungen übersetzen.</t>
-  </si>
-  <si>
-    <t>Welches Ziel hat STOCKMEIER in Bezug auf Sicherheit formuliert?</t>
-  </si>
-  <si>
-    <t>Alle Sicherheitsschulungen durch Plakate ersetzen</t>
-  </si>
-  <si>
-    <t>Null arbeitsbedingte Unfälle</t>
-  </si>
-  <si>
-    <t>Nur Unfälle in Büros reduzieren</t>
-  </si>
-  <si>
-    <t>Unfälle akzeptieren, wenn Produktionsziele erreicht werden</t>
-  </si>
-  <si>
-    <t>Der Bericht nennt das Ziel von null arbeitsbedingten Unfällen und null gesundheitsschädlichen Auswirkungen. Beispiele von STOCKMEIER machen das SDG konkret und zeigen, wie Initiativen der Gruppe mit globalen Zielen verbunden sind.</t>
-  </si>
-  <si>
     <t>Quelle est l'idée principale de l'ODD 3 – Bonne santé et bien-être ?</t>
   </si>
   <si>
@@ -366,13 +288,106 @@
   </si>
   <si>
     <t>W raporcie określono ambicję osiągnięcia zerowej liczby wypadków związanych z pracą oraz zerowego szkodliwego wpływu na zdrowie. Przykłady ze STOCKMEIER konkretyzują SDG i pokazują, jak inicjatywy Grupy łączą się z globalnymi celami.</t>
+  </si>
+  <si>
+    <t>What does sustainability in everyday work mean most of all?</t>
+  </si>
+  <si>
+    <t>Single choice</t>
+  </si>
+  <si>
+    <t>Only large projects matter, not small daily decisions.</t>
+  </si>
+  <si>
+    <t>Sustainability is an ongoing process that we can support every day.</t>
+  </si>
+  <si>
+    <t>Sustainability only concerns environmental departments and managers.</t>
+  </si>
+  <si>
+    <t>Sustainability is a topic for later, not for today's work.</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>The report describes sustainability as a daily path, not a one-time goal.</t>
+  </si>
+  <si>
+    <t>multiple</t>
+  </si>
+  <si>
+    <t>Which goals fit the “Zero in Focus” idea?</t>
+  </si>
+  <si>
+    <t>Multiple choice</t>
+  </si>
+  <si>
+    <t>Zero CO₂ emissions</t>
+  </si>
+  <si>
+    <t>Zero accidents at work</t>
+  </si>
+  <si>
+    <t>Zero tolerance for unethical behaviour</t>
+  </si>
+  <si>
+    <t>Zero training</t>
+  </si>
+  <si>
+    <t>0,1,2</t>
+  </si>
+  <si>
+    <t>The idea combines climate, safety and integrity. Training is not a “Zero” goal.</t>
+  </si>
+  <si>
+    <t>Was bedeutet Nachhaltigkeit im Arbeitsalltag vor allem?</t>
+  </si>
+  <si>
+    <t>Einfachauswahl</t>
+  </si>
+  <si>
+    <t>Nur große Projekte zählen, nicht kleine tägliche Entscheidungen.</t>
+  </si>
+  <si>
+    <t>Nachhaltigkeit ist ein fortlaufender Prozess, den wir jeden Tag unterstützen können.</t>
+  </si>
+  <si>
+    <t>Nachhaltigkeit betrifft nur Umweltabteilungen und Führungskräfte.</t>
+  </si>
+  <si>
+    <t>Nachhaltigkeit ist ein Thema für später, nicht für die heutige Arbeit.</t>
+  </si>
+  <si>
+    <t>Der Bericht beschreibt Nachhaltigkeit als einen täglichen Weg und nicht als einmaliges Ziel.</t>
+  </si>
+  <si>
+    <t>Welche Ziele passen zur Idee „Zero in Focus“?</t>
+  </si>
+  <si>
+    <t>Mehrfachauswahl</t>
+  </si>
+  <si>
+    <t>Null CO₂-Emissionen</t>
+  </si>
+  <si>
+    <t>Null Arbeitsunfälle</t>
+  </si>
+  <si>
+    <t>Null Toleranz gegenüber unethischem Verhalten</t>
+  </si>
+  <si>
+    <t>Null Schulungen</t>
+  </si>
+  <si>
+    <t>Die Idee verbindet Klima, Sicherheit und Integrität. Schulungen sind kein „Zero“-Ziel.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -384,16 +399,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -440,7 +445,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -468,11 +473,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD8D8D4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -480,58 +494,268 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="51">
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
+  <dxfs count="63">
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top/>
+        <bottom style="thin">
+          <color rgb="FFD8D8D4"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <alignment wrapText="1"/>
@@ -969,6 +1193,9 @@
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -986,15 +1213,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Questions" displayName="Questions" ref="A1:J3">
   <autoFilter ref="A1:J3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="type"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="question"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="note"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="option1"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="option2"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="option3"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="option4"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="correct"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="explanation"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="type" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="question" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="note" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="option1" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="option2" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="option3" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="option4" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="correct" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="explanation" dataDxfId="9"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Comments ZF"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1002,19 +1229,19 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F33C372F-7DF1-44B8-A553-F96162E20FF6}" name="Questions_NL" displayName="Questions_NL" ref="A1:J3" totalsRowShown="0" headerRowDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F33C372F-7DF1-44B8-A553-F96162E20FF6}" name="Questions_NL" displayName="Questions_NL" ref="A1:J3" totalsRowShown="0" headerRowDxfId="61">
   <autoFilter ref="A1:J3" xr:uid="{F33C372F-7DF1-44B8-A553-F96162E20FF6}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{8768A190-4619-4E99-A1FB-E085A0691535}" name="type"/>
-    <tableColumn id="2" xr3:uid="{138753B1-3E1C-449D-94EC-F0C2EEB45A70}" name="question" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{138753B1-3E1C-449D-94EC-F0C2EEB45A70}" name="question" dataDxfId="60"/>
     <tableColumn id="3" xr3:uid="{FED00481-A20D-41CA-B9AD-1BEC5A6526F9}" name="note"/>
-    <tableColumn id="4" xr3:uid="{4C97B040-4120-4B99-933B-CBD2000E9533}" name="option1" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{2A6AFBEF-0DA7-467B-A43E-90728CFDE3FA}" name="option2" dataDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{C01A211B-00E9-4EAC-B1E5-E7E8A3AC81EB}" name="option3" dataDxfId="46"/>
-    <tableColumn id="7" xr3:uid="{AD151611-2D1E-44FE-BA77-0142DB062F48}" name="option4" dataDxfId="45"/>
+    <tableColumn id="4" xr3:uid="{4C97B040-4120-4B99-933B-CBD2000E9533}" name="option1" dataDxfId="59"/>
+    <tableColumn id="5" xr3:uid="{2A6AFBEF-0DA7-467B-A43E-90728CFDE3FA}" name="option2" dataDxfId="58"/>
+    <tableColumn id="6" xr3:uid="{C01A211B-00E9-4EAC-B1E5-E7E8A3AC81EB}" name="option3" dataDxfId="57"/>
+    <tableColumn id="7" xr3:uid="{AD151611-2D1E-44FE-BA77-0142DB062F48}" name="option4" dataDxfId="56"/>
     <tableColumn id="8" xr3:uid="{7E796F1C-08BD-41F7-8EAA-7AE75851648A}" name="correct"/>
-    <tableColumn id="9" xr3:uid="{71BF8262-57EB-411D-86D6-D11A0BCDCFA5}" name="explanation" dataDxfId="44"/>
-    <tableColumn id="10" xr3:uid="{1E13442E-16C8-44FA-B52D-99CDBBFE4D11}" name="Comments ZF" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{71BF8262-57EB-411D-86D6-D11A0BCDCFA5}" name="explanation" dataDxfId="55"/>
+    <tableColumn id="10" xr3:uid="{1E13442E-16C8-44FA-B52D-99CDBBFE4D11}" name="Comments ZF" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1025,34 +1252,34 @@
   <autoFilter ref="A1:J3" xr:uid="{0443C156-3373-4BEF-9D5B-BE15850933BA}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{F437D6E2-54A8-46CF-B6AA-72B1DDDBD98E}" name="type"/>
-    <tableColumn id="2" xr3:uid="{952F0744-7AAB-463E-BCD7-2E26EA55F0B5}" name="question" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{952F0744-7AAB-463E-BCD7-2E26EA55F0B5}" name="question" dataDxfId="53"/>
     <tableColumn id="3" xr3:uid="{2B1FC043-0C02-4B8E-9EEB-67C6FA02E0F8}" name="note"/>
-    <tableColumn id="4" xr3:uid="{EAD83E31-505A-42DC-942F-F9E48303E96B}" name="option1" dataDxfId="41"/>
-    <tableColumn id="5" xr3:uid="{C9E5F8DA-09FA-45D4-B2F9-7D4E6C797F1B}" name="option2" dataDxfId="40"/>
-    <tableColumn id="6" xr3:uid="{4F227AFF-14FF-495C-A638-834DE2F2F0F1}" name="option3" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{03B75AA8-AED7-4944-9BBB-FA1CDA99CE3C}" name="option4" dataDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{EAD83E31-505A-42DC-942F-F9E48303E96B}" name="option1" dataDxfId="52"/>
+    <tableColumn id="5" xr3:uid="{C9E5F8DA-09FA-45D4-B2F9-7D4E6C797F1B}" name="option2" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{4F227AFF-14FF-495C-A638-834DE2F2F0F1}" name="option3" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{03B75AA8-AED7-4944-9BBB-FA1CDA99CE3C}" name="option4" dataDxfId="49"/>
     <tableColumn id="8" xr3:uid="{A9DB8E5B-B50B-451E-80E7-BC3C1E2EB942}" name="correct"/>
-    <tableColumn id="9" xr3:uid="{596E4A30-D592-45A2-9BA6-909C7233F36E}" name="explanation" dataDxfId="37"/>
-    <tableColumn id="10" xr3:uid="{E0D67ADC-A9CC-4A55-ABB2-99CF33216FD1}" name="Comments ZF" dataDxfId="36"/>
+    <tableColumn id="9" xr3:uid="{596E4A30-D592-45A2-9BA6-909C7233F36E}" name="explanation" dataDxfId="48"/>
+    <tableColumn id="10" xr3:uid="{E0D67ADC-A9CC-4A55-ABB2-99CF33216FD1}" name="Comments ZF" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{44E0FAA6-8BD7-4759-AAA3-94BECD54F540}" name="Questions_PL" displayName="Questions_PL" ref="A1:J3" totalsRowShown="0" headerRowDxfId="35" dataDxfId="33" headerRowBorderDxfId="34" tableBorderDxfId="32" totalsRowBorderDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{44E0FAA6-8BD7-4759-AAA3-94BECD54F540}" name="Questions_PL" displayName="Questions_PL" ref="A1:J3" totalsRowShown="0" headerRowDxfId="46" dataDxfId="44" headerRowBorderDxfId="45" tableBorderDxfId="43" totalsRowBorderDxfId="42">
   <autoFilter ref="A1:J3" xr:uid="{44E0FAA6-8BD7-4759-AAA3-94BECD54F540}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{B8E1CEFB-D4F5-4454-8EE2-4CC13B41524D}" name="type" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{0B3BB530-19FC-4EF1-8906-128ED72B0CF4}" name="question" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{A026DC58-89E8-41A8-87BF-377C94896F3B}" name="note" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{E52F3421-7180-4A31-AD6A-7C5921781982}" name="option1" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{50128664-5FE2-4CA5-B1A5-9B8B853A2B64}" name="option2" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{57AC2722-D37E-4A00-8697-571E06CE666D}" name="option3" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{6127D6A3-5DD7-4DBA-B556-18BCAA69EB40}" name="option4" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{8345AB07-2F86-429A-A477-BB8EC49876B0}" name="correct" dataDxfId="23"/>
-    <tableColumn id="9" xr3:uid="{E51614FA-9BED-41B9-8BFE-5ED5998D9CA0}" name="explanation" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{0BD74B70-C4EA-40E7-8E13-D86793442E46}" name="Comments ZF" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{B8E1CEFB-D4F5-4454-8EE2-4CC13B41524D}" name="type" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{0B3BB530-19FC-4EF1-8906-128ED72B0CF4}" name="question" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{A026DC58-89E8-41A8-87BF-377C94896F3B}" name="note" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{E52F3421-7180-4A31-AD6A-7C5921781982}" name="option1" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{50128664-5FE2-4CA5-B1A5-9B8B853A2B64}" name="option2" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{57AC2722-D37E-4A00-8697-571E06CE666D}" name="option3" dataDxfId="36"/>
+    <tableColumn id="7" xr3:uid="{6127D6A3-5DD7-4DBA-B556-18BCAA69EB40}" name="option4" dataDxfId="35"/>
+    <tableColumn id="8" xr3:uid="{8345AB07-2F86-429A-A477-BB8EC49876B0}" name="correct" dataDxfId="34"/>
+    <tableColumn id="9" xr3:uid="{E51614FA-9BED-41B9-8BFE-5ED5998D9CA0}" name="explanation" dataDxfId="33"/>
+    <tableColumn id="10" xr3:uid="{0BD74B70-C4EA-40E7-8E13-D86793442E46}" name="Comments ZF" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1063,15 +1290,15 @@
   <autoFilter ref="A1:J3" xr:uid="{24328404-240E-47C6-99B4-84D4666E487C}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{D28DA00C-53DD-41D8-A3BF-DB525A0D4771}" name="type"/>
-    <tableColumn id="2" xr3:uid="{175F879F-6B11-4B9A-8454-1120A2D79E3F}" name="question" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{175F879F-6B11-4B9A-8454-1120A2D79E3F}" name="question" dataDxfId="31"/>
     <tableColumn id="3" xr3:uid="{F21BF042-E407-4DB9-A79D-DA0E245869A5}" name="note"/>
-    <tableColumn id="4" xr3:uid="{619CB46F-4592-4C56-A69F-68EB3309A9BB}" name="option1" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{50FBD72E-8E38-49CB-B7A5-F14034CD6617}" name="option2" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{26B75C25-0F86-4BC5-A8FD-E52ECDA5672E}" name="option3" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{A923C1B9-61C5-420B-883C-04A0A11B7BC5}" name="option4" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{619CB46F-4592-4C56-A69F-68EB3309A9BB}" name="option1" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{50FBD72E-8E38-49CB-B7A5-F14034CD6617}" name="option2" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{26B75C25-0F86-4BC5-A8FD-E52ECDA5672E}" name="option3" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{A923C1B9-61C5-420B-883C-04A0A11B7BC5}" name="option4" dataDxfId="27"/>
     <tableColumn id="8" xr3:uid="{6F0FFD5B-A111-4E68-B09A-F9C8C262B0AE}" name="correct"/>
-    <tableColumn id="9" xr3:uid="{2ABE4738-C112-4F9E-8A03-64A555F8DFCB}" name="explanation" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{6886EBCC-E8F2-4112-BF52-377F836CE96C}" name="Comments ZF" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{2ABE4738-C112-4F9E-8A03-64A555F8DFCB}" name="explanation" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{6886EBCC-E8F2-4112-BF52-377F836CE96C}" name="Comments ZF" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1082,15 +1309,15 @@
   <autoFilter ref="A1:J3" xr:uid="{69487D5A-D6BB-406F-B006-C23DC0801576}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{11EBFC79-7169-44C9-98FF-AEAD54A3F4CF}" name="type"/>
-    <tableColumn id="2" xr3:uid="{D15870D6-4160-450D-8A48-A45F378320C5}" name="question" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{D15870D6-4160-450D-8A48-A45F378320C5}" name="question" dataDxfId="24"/>
     <tableColumn id="3" xr3:uid="{5BC96237-C15E-4AF1-BB12-192ED4C16B04}" name="note"/>
-    <tableColumn id="4" xr3:uid="{A7B78417-59DE-4F90-81A8-EF0636F85EF1}" name="option1" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{C10D44DD-CD72-49D7-AF76-3B9DBCC1FB72}" name="option2" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{D24F9622-47A3-40CF-8336-5D9ABAFAB985}" name="option3" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{E354F182-1976-4AA1-88B5-B44C580AD1F1}" name="option4" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{A7B78417-59DE-4F90-81A8-EF0636F85EF1}" name="option1" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{C10D44DD-CD72-49D7-AF76-3B9DBCC1FB72}" name="option2" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{D24F9622-47A3-40CF-8336-5D9ABAFAB985}" name="option3" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{E354F182-1976-4AA1-88B5-B44C580AD1F1}" name="option4" dataDxfId="20"/>
     <tableColumn id="8" xr3:uid="{E6194F33-38E1-4D8F-AC4B-43D3240E8F29}" name="correct"/>
-    <tableColumn id="9" xr3:uid="{52ABFCD8-07EF-429C-B7F4-3C69747A12F2}" name="explanation" dataDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{6C0169E4-F1E8-4B5D-BE55-5684B57CF5ED}" name="Comments ZF" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{52ABFCD8-07EF-429C-B7F4-3C69747A12F2}" name="explanation" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{6C0169E4-F1E8-4B5D-BE55-5684B57CF5ED}" name="Comments ZF" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1100,16 +1327,16 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{03F5E4B0-1EE4-4A96-B063-5B136C1A51C8}" name="Questions_GE" displayName="Questions_GE" ref="A1:J3">
   <autoFilter ref="A1:J3" xr:uid="{03F5E4B0-1EE4-4A96-B063-5B136C1A51C8}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{6EBC16CA-B01C-4958-B5F0-385E02F2076F}" name="type"/>
-    <tableColumn id="2" xr3:uid="{17A07ACE-7C03-46F0-BB3C-0E2AEBB60E87}" name="question" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{21C55411-3486-4BC8-BDEB-1355F960228C}" name="note"/>
+    <tableColumn id="1" xr3:uid="{6EBC16CA-B01C-4958-B5F0-385E02F2076F}" name="type" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{17A07ACE-7C03-46F0-BB3C-0E2AEBB60E87}" name="question" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{21C55411-3486-4BC8-BDEB-1355F960228C}" name="note" dataDxfId="6"/>
     <tableColumn id="4" xr3:uid="{3DC4C62B-B6B5-4550-B418-91D15C90EF11}" name="option1" dataDxfId="5"/>
     <tableColumn id="5" xr3:uid="{A93353C8-8D88-4219-903B-30B1C42FF339}" name="option2" dataDxfId="4"/>
     <tableColumn id="6" xr3:uid="{FB6C5E79-096F-4610-A1AF-1E2713100CE6}" name="option3" dataDxfId="3"/>
     <tableColumn id="7" xr3:uid="{C83EC64E-DF84-427F-92DC-1D91223EB6AE}" name="option4" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{6B2FC0C7-D58D-4EEE-9847-3B9CF8F4FCCA}" name="correct"/>
-    <tableColumn id="9" xr3:uid="{C2B6DEC7-7756-44AE-8BB4-CBF8A804D904}" name="explanation" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{62EB005F-AEC9-4EB3-B430-68004B533DA8}" name="Comments ZF" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{6B2FC0C7-D58D-4EEE-9847-3B9CF8F4FCCA}" name="correct" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{C2B6DEC7-7756-44AE-8BB4-CBF8A804D904}" name="explanation" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{62EB005F-AEC9-4EB3-B430-68004B533DA8}" name="Comments ZF" dataDxfId="62"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1445,67 +1672,67 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="2">
-        <v>1</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="2">
-        <v>2</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>24</v>
+      <c r="A3" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>98</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1566,64 +1793,64 @@
       <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>25</v>
+      <c r="B2" s="3" t="s">
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>30</v>
+        <v>13</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>32</v>
+      <c r="I2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>33</v>
+      <c r="B3" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>37</v>
+        <v>13</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>24</v>
       </c>
       <c r="H3">
         <v>2</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>32</v>
+      <c r="I3" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1684,64 +1911,64 @@
       <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>52</v>
+      <c r="B2" s="3" t="s">
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>57</v>
+        <v>27</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>59</v>
+      <c r="I2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>60</v>
+      <c r="B3" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>64</v>
+        <v>27</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>38</v>
       </c>
       <c r="H3">
         <v>2</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>59</v>
+      <c r="I3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1767,99 +1994,99 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="9" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="H2" s="6">
+      <c r="B2" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H2" s="4">
         <v>1</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>101</v>
+      <c r="I2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="75" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="H3" s="9">
+      <c r="B3" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="H3" s="7">
         <v>2</v>
       </c>
-      <c r="I3" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>101</v>
+      <c r="I3" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1920,64 +2147,64 @@
       <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>66</v>
+      <c r="B2" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>71</v>
+        <v>41</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>73</v>
+      <c r="I2" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>74</v>
+      <c r="B3" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>78</v>
+        <v>41</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>52</v>
       </c>
       <c r="H3">
         <v>2</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>73</v>
+      <c r="I3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -2038,64 +2265,64 @@
       <c r="A2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>80</v>
+      <c r="B2" s="3" t="s">
+        <v>54</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>85</v>
+        <v>55</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>59</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>87</v>
+      <c r="I2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>88</v>
+      <c r="B3" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>81</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>92</v>
+        <v>55</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>66</v>
       </c>
       <c r="H3">
         <v>2</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>87</v>
+      <c r="I3" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -2152,68 +2379,68 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="H2" s="2">
-        <v>1</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>45</v>
+      <c r="B2" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>105</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="H3" s="2">
-        <v>2</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>51</v>
+    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -2225,16 +2452,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2aad7df3-4ab7-4daa-980d-cf7206357ce9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101006B71C29808C7F3499BFFC3671560B6FA" ma:contentTypeVersion="8" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="e4f9e1976b194f932bebfa03c600f49f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2aad7df3-4ab7-4daa-980d-cf7206357ce9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8d33a1b74cd678b812bcd025038ca576" ns2:_="">
     <xsd:import namespace="2aad7df3-4ab7-4daa-980d-cf7206357ce9"/>
@@ -2398,6 +2615,16 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2aad7df3-4ab7-4daa-980d-cf7206357ce9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2408,16 +2635,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A947F87A-A862-469B-80AB-EC8D5B706ABA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2aad7df3-4ab7-4daa-980d-cf7206357ce9"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{052D775B-35AE-4D8C-85B8-39FE1C3B4BBC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2435,6 +2652,16 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A947F87A-A862-469B-80AB-EC8D5B706ABA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2aad7df3-4ab7-4daa-980d-cf7206357ce9"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79A12AD6-4D28-47C9-A756-6744BC5075CA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Test to fix questions (layout to text)
</commit_message>
<xml_diff>
--- a/Questions - Round 1.xlsx
+++ b/Questions - Round 1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://innochemnv-my.sharepoint.com/personal/zander_fias_innochem_be/Documents/OneDrive_1_25-9-2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cafnzholding-my.sharepoint.com/personal/thom_van_dusschoten_synerlogic_nl/Documents/Documenten/GitHub/Sustainability-quiz-TEST/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="119" documentId="11_DC4634EEB09B7631DD1D459FDEF3484CE4F5FC66" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46E1F90F-679A-4B57-A7C5-A373B94A5194}"/>
+  <xr:revisionPtr revIDLastSave="127" documentId="11_DC4634EEB09B7631DD1D459FDEF3484CE4F5FC66" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F19F1512-86DB-4AD0-AA3F-331DCE8392A2}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EN" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="465">
   <si>
     <t>type</t>
   </si>
@@ -450,36 +450,6 @@
   </si>
   <si>
     <t>Lichaamsbeweging, rust en om steun vragen dragen bij aan welzijn. Persoonlijke gewoonten zijn belangrijk omdat veel kleine keuzes betekenisvol worden wanneer veel mensen ze herhalen.</t>
-  </si>
-  <si>
-    <t>Column1</t>
-  </si>
-  <si>
-    <t>Column2</t>
-  </si>
-  <si>
-    <t>Column3</t>
-  </si>
-  <si>
-    <t>Column4</t>
-  </si>
-  <si>
-    <t>Column5</t>
-  </si>
-  <si>
-    <t>Column6</t>
-  </si>
-  <si>
-    <t>Column7</t>
-  </si>
-  <si>
-    <t>Column8</t>
-  </si>
-  <si>
-    <t>Column9</t>
-  </si>
-  <si>
-    <t>Column10</t>
   </si>
   <si>
     <t>Was ist die zentrale Idee hinter SDG 3 – Gesundheit und Wohlergehen?</t>
@@ -1582,7 +1552,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1626,11 +1596,30 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="50">
+  <dxfs count="57">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
     <dxf>
       <alignment wrapText="1"/>
     </dxf>
@@ -1638,25 +1627,126 @@
       <alignment wrapText="1"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <alignment wrapText="1"/>
     </dxf>
     <dxf>
       <alignment wrapText="1"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <alignment wrapText="1"/>
     </dxf>
     <dxf>
       <alignment wrapText="1"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <alignment wrapText="1"/>
     </dxf>
     <dxf>
       <alignment wrapText="1"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F4E78"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <alignment wrapText="1"/>
@@ -1779,10 +1869,44 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <name val="Calibri"/>
         <family val="2"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -1830,74 +1954,6 @@
       </border>
     </dxf>
     <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1960,37 +2016,6 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -2077,10 +2102,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Questions" displayName="Questions" ref="A1:J11">
   <autoFilter ref="A1:J11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
@@ -2092,7 +2113,7 @@
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="option2"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="option3"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="option4"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="correct"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="correct" dataDxfId="16"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="explanation"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Comments ZF"/>
   </tableColumns>
@@ -2101,19 +2122,19 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F33C372F-7DF1-44B8-A553-F96162E20FF6}" name="Questions_NL" displayName="Questions_NL" ref="A1:J11" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F33C372F-7DF1-44B8-A553-F96162E20FF6}" name="Questions_NL" displayName="Questions_NL" ref="A1:J11" totalsRowShown="0" headerRowDxfId="15">
   <autoFilter ref="A1:J11" xr:uid="{F33C372F-7DF1-44B8-A553-F96162E20FF6}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{8768A190-4619-4E99-A1FB-E085A0691535}" name="Column1"/>
-    <tableColumn id="2" xr3:uid="{138753B1-3E1C-449D-94EC-F0C2EEB45A70}" name="Column2" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{FED00481-A20D-41CA-B9AD-1BEC5A6526F9}" name="Column3"/>
-    <tableColumn id="4" xr3:uid="{4C97B040-4120-4B99-933B-CBD2000E9533}" name="Column4" dataDxfId="33"/>
-    <tableColumn id="5" xr3:uid="{2A6AFBEF-0DA7-467B-A43E-90728CFDE3FA}" name="Column5" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{C01A211B-00E9-4EAC-B1E5-E7E8A3AC81EB}" name="Column6" dataDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{AD151611-2D1E-44FE-BA77-0142DB062F48}" name="Column7" dataDxfId="30"/>
-    <tableColumn id="8" xr3:uid="{7E796F1C-08BD-41F7-8EAA-7AE75851648A}" name="Column8"/>
-    <tableColumn id="9" xr3:uid="{71BF8262-57EB-411D-86D6-D11A0BCDCFA5}" name="Column9" dataDxfId="29"/>
-    <tableColumn id="10" xr3:uid="{1E13442E-16C8-44FA-B52D-99CDBBFE4D11}" name="Column10" dataDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{8768A190-4619-4E99-A1FB-E085A0691535}" name="type"/>
+    <tableColumn id="2" xr3:uid="{138753B1-3E1C-449D-94EC-F0C2EEB45A70}" name="question" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{FED00481-A20D-41CA-B9AD-1BEC5A6526F9}" name="note"/>
+    <tableColumn id="4" xr3:uid="{4C97B040-4120-4B99-933B-CBD2000E9533}" name="option1" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{2A6AFBEF-0DA7-467B-A43E-90728CFDE3FA}" name="option2" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{C01A211B-00E9-4EAC-B1E5-E7E8A3AC81EB}" name="option3" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{AD151611-2D1E-44FE-BA77-0142DB062F48}" name="option4" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{7E796F1C-08BD-41F7-8EAA-7AE75851648A}" name="correct" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{71BF8262-57EB-411D-86D6-D11A0BCDCFA5}" name="explanation" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{1E13442E-16C8-44FA-B52D-99CDBBFE4D11}" name="Comments ZF" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2124,34 +2145,34 @@
   <autoFilter ref="A1:J11" xr:uid="{0443C156-3373-4BEF-9D5B-BE15850933BA}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{F437D6E2-54A8-46CF-B6AA-72B1DDDBD98E}" name="type"/>
-    <tableColumn id="2" xr3:uid="{952F0744-7AAB-463E-BCD7-2E26EA55F0B5}" name="question" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{952F0744-7AAB-463E-BCD7-2E26EA55F0B5}" name="question" dataDxfId="39"/>
     <tableColumn id="3" xr3:uid="{2B1FC043-0C02-4B8E-9EEB-67C6FA02E0F8}" name="note"/>
-    <tableColumn id="4" xr3:uid="{EAD83E31-505A-42DC-942F-F9E48303E96B}" name="option1" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{C9E5F8DA-09FA-45D4-B2F9-7D4E6C797F1B}" name="option2" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{4F227AFF-14FF-495C-A638-834DE2F2F0F1}" name="option3" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{03B75AA8-AED7-4944-9BBB-FA1CDA99CE3C}" name="option4" dataDxfId="23"/>
-    <tableColumn id="8" xr3:uid="{A9DB8E5B-B50B-451E-80E7-BC3C1E2EB942}" name="correct"/>
-    <tableColumn id="9" xr3:uid="{596E4A30-D592-45A2-9BA6-909C7233F36E}" name="explanation" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{E0D67ADC-A9CC-4A55-ABB2-99CF33216FD1}" name="Comments ZF" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{EAD83E31-505A-42DC-942F-F9E48303E96B}" name="option1" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{C9E5F8DA-09FA-45D4-B2F9-7D4E6C797F1B}" name="option2" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{4F227AFF-14FF-495C-A638-834DE2F2F0F1}" name="option3" dataDxfId="36"/>
+    <tableColumn id="7" xr3:uid="{03B75AA8-AED7-4944-9BBB-FA1CDA99CE3C}" name="option4" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{A9DB8E5B-B50B-451E-80E7-BC3C1E2EB942}" name="correct" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{596E4A30-D592-45A2-9BA6-909C7233F36E}" name="explanation" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{E0D67ADC-A9CC-4A55-ABB2-99CF33216FD1}" name="Comments ZF" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{44E0FAA6-8BD7-4759-AAA3-94BECD54F540}" name="Questions_PL" displayName="Questions_PL" ref="A1:J11" totalsRowShown="0" headerRowDxfId="49" dataDxfId="47" headerRowBorderDxfId="48" tableBorderDxfId="46" totalsRowBorderDxfId="45">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{44E0FAA6-8BD7-4759-AAA3-94BECD54F540}" name="Questions_PL" displayName="Questions_PL" ref="A1:J11" totalsRowShown="0" headerRowDxfId="56" dataDxfId="54" headerRowBorderDxfId="55" tableBorderDxfId="53" totalsRowBorderDxfId="52">
   <autoFilter ref="A1:J11" xr:uid="{44E0FAA6-8BD7-4759-AAA3-94BECD54F540}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{B8E1CEFB-D4F5-4454-8EE2-4CC13B41524D}" name="type" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{0B3BB530-19FC-4EF1-8906-128ED72B0CF4}" name="question" dataDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{A026DC58-89E8-41A8-87BF-377C94896F3B}" name="note" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{E52F3421-7180-4A31-AD6A-7C5921781982}" name="option1" dataDxfId="41"/>
-    <tableColumn id="5" xr3:uid="{50128664-5FE2-4CA5-B1A5-9B8B853A2B64}" name="option2" dataDxfId="40"/>
-    <tableColumn id="6" xr3:uid="{57AC2722-D37E-4A00-8697-571E06CE666D}" name="option3" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{6127D6A3-5DD7-4DBA-B556-18BCAA69EB40}" name="option4" dataDxfId="38"/>
-    <tableColumn id="8" xr3:uid="{8345AB07-2F86-429A-A477-BB8EC49876B0}" name="correct" dataDxfId="37"/>
-    <tableColumn id="9" xr3:uid="{E51614FA-9BED-41B9-8BFE-5ED5998D9CA0}" name="explanation" dataDxfId="36"/>
-    <tableColumn id="10" xr3:uid="{0BD74B70-C4EA-40E7-8E13-D86793442E46}" name="Comments ZF" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{B8E1CEFB-D4F5-4454-8EE2-4CC13B41524D}" name="type" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{0B3BB530-19FC-4EF1-8906-128ED72B0CF4}" name="question" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{A026DC58-89E8-41A8-87BF-377C94896F3B}" name="note" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{E52F3421-7180-4A31-AD6A-7C5921781982}" name="option1" dataDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{50128664-5FE2-4CA5-B1A5-9B8B853A2B64}" name="option2" dataDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{57AC2722-D37E-4A00-8697-571E06CE666D}" name="option3" dataDxfId="46"/>
+    <tableColumn id="7" xr3:uid="{6127D6A3-5DD7-4DBA-B556-18BCAA69EB40}" name="option4" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{8345AB07-2F86-429A-A477-BB8EC49876B0}" name="correct" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{E51614FA-9BED-41B9-8BFE-5ED5998D9CA0}" name="explanation" dataDxfId="18"/>
+    <tableColumn id="10" xr3:uid="{0BD74B70-C4EA-40E7-8E13-D86793442E46}" name="Comments ZF" dataDxfId="45"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2162,15 +2183,15 @@
   <autoFilter ref="A1:J11" xr:uid="{24328404-240E-47C6-99B4-84D4666E487C}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{D28DA00C-53DD-41D8-A3BF-DB525A0D4771}" name="type"/>
-    <tableColumn id="2" xr3:uid="{175F879F-6B11-4B9A-8454-1120A2D79E3F}" name="question" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{175F879F-6B11-4B9A-8454-1120A2D79E3F}" name="question" dataDxfId="34"/>
     <tableColumn id="3" xr3:uid="{F21BF042-E407-4DB9-A79D-DA0E245869A5}" name="note"/>
-    <tableColumn id="4" xr3:uid="{619CB46F-4592-4C56-A69F-68EB3309A9BB}" name="option1" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{50FBD72E-8E38-49CB-B7A5-F14034CD6617}" name="option2" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{26B75C25-0F86-4BC5-A8FD-E52ECDA5672E}" name="option3" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{A923C1B9-61C5-420B-883C-04A0A11B7BC5}" name="option4" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{6F0FFD5B-A111-4E68-B09A-F9C8C262B0AE}" name="correct"/>
-    <tableColumn id="9" xr3:uid="{2ABE4738-C112-4F9E-8A03-64A555F8DFCB}" name="explanation" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{6886EBCC-E8F2-4112-BF52-377F836CE96C}" name="Comments ZF" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{619CB46F-4592-4C56-A69F-68EB3309A9BB}" name="option1" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{50FBD72E-8E38-49CB-B7A5-F14034CD6617}" name="option2" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{26B75C25-0F86-4BC5-A8FD-E52ECDA5672E}" name="option3" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{A923C1B9-61C5-420B-883C-04A0A11B7BC5}" name="option4" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{6F0FFD5B-A111-4E68-B09A-F9C8C262B0AE}" name="correct" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{2ABE4738-C112-4F9E-8A03-64A555F8DFCB}" name="explanation" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{6886EBCC-E8F2-4112-BF52-377F836CE96C}" name="Comments ZF" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2181,15 +2202,15 @@
   <autoFilter ref="A1:J11" xr:uid="{69487D5A-D6BB-406F-B006-C23DC0801576}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{11EBFC79-7169-44C9-98FF-AEAD54A3F4CF}" name="type"/>
-    <tableColumn id="2" xr3:uid="{D15870D6-4160-450D-8A48-A45F378320C5}" name="question" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{D15870D6-4160-450D-8A48-A45F378320C5}" name="question" dataDxfId="29"/>
     <tableColumn id="3" xr3:uid="{5BC96237-C15E-4AF1-BB12-192ED4C16B04}" name="note"/>
-    <tableColumn id="4" xr3:uid="{A7B78417-59DE-4F90-81A8-EF0636F85EF1}" name="option1" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{C10D44DD-CD72-49D7-AF76-3B9DBCC1FB72}" name="option2" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{D24F9622-47A3-40CF-8336-5D9ABAFAB985}" name="option3" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{E354F182-1976-4AA1-88B5-B44C580AD1F1}" name="option4" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{E6194F33-38E1-4D8F-AC4B-43D3240E8F29}" name="correct"/>
-    <tableColumn id="9" xr3:uid="{52ABFCD8-07EF-429C-B7F4-3C69747A12F2}" name="explanation" dataDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{6C0169E4-F1E8-4B5D-BE55-5684B57CF5ED}" name="Comments ZF" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{A7B78417-59DE-4F90-81A8-EF0636F85EF1}" name="option1" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{C10D44DD-CD72-49D7-AF76-3B9DBCC1FB72}" name="option2" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{D24F9622-47A3-40CF-8336-5D9ABAFAB985}" name="option3" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{E354F182-1976-4AA1-88B5-B44C580AD1F1}" name="option4" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{E6194F33-38E1-4D8F-AC4B-43D3240E8F29}" name="correct" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{52ABFCD8-07EF-429C-B7F4-3C69747A12F2}" name="explanation" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{6C0169E4-F1E8-4B5D-BE55-5684B57CF5ED}" name="Comments ZF" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2200,15 +2221,15 @@
   <autoFilter ref="A1:J11" xr:uid="{03F5E4B0-1EE4-4A96-B063-5B136C1A51C8}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{6EBC16CA-B01C-4958-B5F0-385E02F2076F}" name="type"/>
-    <tableColumn id="2" xr3:uid="{17A07ACE-7C03-46F0-BB3C-0E2AEBB60E87}" name="question" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{17A07ACE-7C03-46F0-BB3C-0E2AEBB60E87}" name="question" dataDxfId="24"/>
     <tableColumn id="3" xr3:uid="{21C55411-3486-4BC8-BDEB-1355F960228C}" name="note"/>
-    <tableColumn id="4" xr3:uid="{3DC4C62B-B6B5-4550-B418-91D15C90EF11}" name="option1" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{A93353C8-8D88-4219-903B-30B1C42FF339}" name="option2" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{FB6C5E79-096F-4610-A1AF-1E2713100CE6}" name="option3" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{C83EC64E-DF84-427F-92DC-1D91223EB6AE}" name="option4" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{6B2FC0C7-D58D-4EEE-9847-3B9CF8F4FCCA}" name="correct"/>
-    <tableColumn id="9" xr3:uid="{C2B6DEC7-7756-44AE-8BB4-CBF8A804D904}" name="explanation" dataDxfId="1"/>
-    <tableColumn id="10" xr3:uid="{62EB005F-AEC9-4EB3-B430-68004B533DA8}" name="Comments ZF" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{3DC4C62B-B6B5-4550-B418-91D15C90EF11}" name="option1" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{A93353C8-8D88-4219-903B-30B1C42FF339}" name="option2" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{FB6C5E79-096F-4610-A1AF-1E2713100CE6}" name="option3" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{C83EC64E-DF84-427F-92DC-1D91223EB6AE}" name="option4" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{6B2FC0C7-D58D-4EEE-9847-3B9CF8F4FCCA}" name="correct" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{C2B6DEC7-7756-44AE-8BB4-CBF8A804D904}" name="explanation" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{62EB005F-AEC9-4EB3-B430-68004B533DA8}" name="Comments ZF" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2500,18 +2521,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="55" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
     <col min="4" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="8" max="8" width="12" style="20" customWidth="1"/>
     <col min="9" max="9" width="75" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2533,7 +2554,7 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="18" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -2543,7 +2564,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2565,7 +2586,7 @@
       <c r="G2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="19">
         <v>1</v>
       </c>
       <c r="I2" s="2" t="s">
@@ -2575,12 +2596,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>19</v>
@@ -2597,7 +2618,7 @@
       <c r="G3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="19">
         <v>2</v>
       </c>
       <c r="I3" s="2" t="s">
@@ -2607,12 +2628,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>461</v>
+        <v>451</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>12</v>
@@ -2629,7 +2650,7 @@
       <c r="G4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="19">
         <v>3</v>
       </c>
       <c r="I4" s="2" t="s">
@@ -2639,12 +2660,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>462</v>
+        <v>452</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>19</v>
@@ -2661,7 +2682,7 @@
       <c r="G5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="19">
         <v>4</v>
       </c>
       <c r="I5" s="2" t="s">
@@ -2671,12 +2692,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>463</v>
+        <v>453</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>19</v>
@@ -2693,7 +2714,7 @@
       <c r="G6" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="19">
         <v>1</v>
       </c>
       <c r="I6" s="2" t="s">
@@ -2703,7 +2724,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
@@ -2725,7 +2746,7 @@
       <c r="G7" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="19">
         <v>2</v>
       </c>
       <c r="I7" s="2" t="s">
@@ -2735,7 +2756,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
@@ -2757,7 +2778,7 @@
       <c r="G8" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="19">
         <v>3</v>
       </c>
       <c r="I8" s="2" t="s">
@@ -2767,7 +2788,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -2789,7 +2810,7 @@
       <c r="G9" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="19">
         <v>4</v>
       </c>
       <c r="I9" s="2" t="s">
@@ -2799,12 +2820,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>464</v>
+        <v>454</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>12</v>
@@ -2821,7 +2842,7 @@
       <c r="G10" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="19">
         <v>1</v>
       </c>
       <c r="I10" s="2" t="s">
@@ -2831,7 +2852,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -2853,7 +2874,7 @@
       <c r="G11" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="19">
         <v>2</v>
       </c>
       <c r="I11" s="2" t="s">
@@ -2874,50 +2895,50 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B227CF05-7239-4F54-B608-C703C72C3BAC}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultColWidth="100" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="100" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.08984375" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.109375" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="7" width="40" customWidth="1"/>
-    <col min="8" max="8" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.77734375" style="20" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="60" customWidth="1"/>
-    <col min="10" max="10" width="19.08984375" customWidth="1"/>
+    <col min="10" max="10" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>136</v>
-      </c>
-      <c r="B1" t="s">
-        <v>137</v>
-      </c>
-      <c r="C1" t="s">
-        <v>138</v>
-      </c>
-      <c r="D1" t="s">
-        <v>139</v>
-      </c>
-      <c r="E1" t="s">
-        <v>140</v>
-      </c>
-      <c r="F1" t="s">
-        <v>141</v>
-      </c>
-      <c r="G1" t="s">
-        <v>142</v>
-      </c>
-      <c r="H1" t="s">
-        <v>143</v>
-      </c>
-      <c r="I1" t="s">
-        <v>144</v>
-      </c>
-      <c r="J1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -2939,7 +2960,7 @@
       <c r="G2" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="20">
         <v>1</v>
       </c>
       <c r="I2" s="5" t="s">
@@ -2949,7 +2970,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -2971,7 +2992,7 @@
       <c r="G3" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="20">
         <v>2</v>
       </c>
       <c r="I3" s="5" t="s">
@@ -2981,7 +3002,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -3003,7 +3024,7 @@
       <c r="G4" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="20">
         <v>3</v>
       </c>
       <c r="I4" s="5" t="s">
@@ -3013,7 +3034,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -3035,7 +3056,7 @@
       <c r="G5" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="20">
         <v>4</v>
       </c>
       <c r="I5" s="5" t="s">
@@ -3045,7 +3066,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -3067,7 +3088,7 @@
       <c r="G6" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="20">
         <v>1</v>
       </c>
       <c r="I6" s="5" t="s">
@@ -3077,7 +3098,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -3099,7 +3120,7 @@
       <c r="G7" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="20">
         <v>2</v>
       </c>
       <c r="I7" s="5" t="s">
@@ -3109,7 +3130,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -3131,7 +3152,7 @@
       <c r="G8" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="20">
         <v>3</v>
       </c>
       <c r="I8" s="5" t="s">
@@ -3141,7 +3162,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -3163,7 +3184,7 @@
       <c r="G9" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="20">
         <v>4</v>
       </c>
       <c r="I9" s="5" t="s">
@@ -3173,7 +3194,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -3195,7 +3216,7 @@
       <c r="G10" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="20">
         <v>1</v>
       </c>
       <c r="I10" s="5" t="s">
@@ -3205,7 +3226,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -3227,7 +3248,7 @@
       <c r="G11" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="20">
         <v>2</v>
       </c>
       <c r="I11" s="5" t="s">
@@ -3248,18 +3269,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1782B8D-F84F-48AC-9C34-ADAF5AFDA9A4}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.08984375" customWidth="1"/>
-    <col min="3" max="3" width="20.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.109375" customWidth="1"/>
+    <col min="3" max="3" width="20.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="7" width="40" customWidth="1"/>
-    <col min="8" max="8" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" style="20" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="60" customWidth="1"/>
-    <col min="10" max="10" width="19.08984375" customWidth="1"/>
+    <col min="10" max="10" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3281,7 +3302,7 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="20" t="s">
         <v>7</v>
       </c>
       <c r="I1" t="s">
@@ -3291,324 +3312,324 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="C2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="H2" s="20">
+        <v>1</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="C3" t="s">
+        <v>209</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E3" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="H3" s="20">
+        <v>2</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="J3" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="H2">
+      <c r="C4" t="s">
+        <v>201</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="H4" s="20">
+        <v>3</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="C5" t="s">
+        <v>209</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="H5" s="20">
+        <v>4</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="C6" t="s">
+        <v>209</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="H6" s="20">
         <v>1</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="C3" t="s">
-        <v>219</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="H3">
+      <c r="I6" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="C7" t="s">
+        <v>201</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="H7" s="20">
         <v>2</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="C4" t="s">
-        <v>211</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="H4">
+      <c r="I7" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="C8" t="s">
+        <v>240</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="H8" s="20">
         <v>3</v>
       </c>
-      <c r="I4" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>231</v>
-      </c>
-      <c r="C5" t="s">
-        <v>219</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="H5">
+      <c r="I8" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="C9" t="s">
+        <v>240</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="H9" s="20">
         <v>4</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="C6" t="s">
-        <v>219</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="H6">
+      <c r="I9" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="C10" t="s">
+        <v>201</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="H10" s="20">
         <v>1</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="C7" t="s">
-        <v>211</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="H7">
+      <c r="I10" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="C11" t="s">
+        <v>201</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="H11" s="20">
         <v>2</v>
       </c>
-      <c r="I7" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="C8" t="s">
-        <v>250</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="E8" s="5" t="s">
+      <c r="I11" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="J11" s="5" t="s">
         <v>252</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="H8">
-        <v>3</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="C9" t="s">
-        <v>250</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="H9">
-        <v>4</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="C10" t="s">
-        <v>211</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>266</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>267</v>
-      </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>268</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="C11" t="s">
-        <v>211</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>271</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>272</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>273</v>
-      </c>
-      <c r="H11">
-        <v>2</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>274</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -3622,18 +3643,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19654F59-BD48-4AA6-AB10-E1FF83EE6625}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.81640625" customWidth="1"/>
-    <col min="2" max="2" width="47.26953125" customWidth="1"/>
-    <col min="3" max="3" width="20.90625" customWidth="1"/>
-    <col min="4" max="7" width="34.54296875" customWidth="1"/>
-    <col min="8" max="8" width="10.90625" customWidth="1"/>
-    <col min="9" max="9" width="56.36328125" customWidth="1"/>
-    <col min="10" max="10" width="18.1796875" customWidth="1"/>
+    <col min="1" max="1" width="11.77734375" customWidth="1"/>
+    <col min="2" max="2" width="47.21875" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" customWidth="1"/>
+    <col min="4" max="7" width="34.5546875" customWidth="1"/>
+    <col min="8" max="8" width="10.88671875" customWidth="1"/>
+    <col min="9" max="9" width="56.33203125" customWidth="1"/>
+    <col min="10" max="10" width="18.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -3665,324 +3686,324 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>465</v>
+        <v>455</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>398</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>399</v>
+      </c>
+      <c r="H2" s="15">
+        <v>1</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>456</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>403</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>404</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>405</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="G3" s="10" t="s">
         <v>406</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="H3" s="16">
+        <v>2</v>
+      </c>
+      <c r="I3" s="9" t="s">
         <v>407</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="J3" s="9" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>457</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>408</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="E4" s="8" t="s">
         <v>409</v>
       </c>
-      <c r="H2" s="6">
+      <c r="F4" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>411</v>
+      </c>
+      <c r="H4" s="15">
+        <v>3</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="H5" s="16">
+        <v>4</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>418</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="H6" s="15">
         <v>1</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>410</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>466</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>412</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>413</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>414</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>415</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>416</v>
-      </c>
-      <c r="H3" s="9">
+      <c r="I6" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>460</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>423</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>425</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="H7" s="16">
         <v>2</v>
       </c>
-      <c r="I3" s="9" t="s">
-        <v>417</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>467</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>405</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>418</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>419</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>420</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>421</v>
-      </c>
-      <c r="H4" s="6">
+      <c r="I7" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>428</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>430</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>431</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="H8" s="15">
         <v>3</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>422</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>468</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>412</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>423</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>424</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>426</v>
-      </c>
-      <c r="H5" s="9">
+      <c r="I8" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>462</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>428</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>434</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>435</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="H9" s="16">
         <v>4</v>
       </c>
-      <c r="I5" s="9" t="s">
-        <v>427</v>
-      </c>
-      <c r="J5" s="9" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>469</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>428</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>429</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>430</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>431</v>
-      </c>
-      <c r="H6" s="6">
+      <c r="I9" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>440</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>441</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>442</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>443</v>
+      </c>
+      <c r="H10" s="15">
         <v>1</v>
       </c>
-      <c r="I6" s="6" t="s">
-        <v>432</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>470</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>405</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>433</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>434</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>435</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>436</v>
-      </c>
-      <c r="H7" s="9">
+      <c r="I10" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>464</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>445</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>446</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>447</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>448</v>
+      </c>
+      <c r="H11" s="17">
         <v>2</v>
       </c>
-      <c r="I7" s="9" t="s">
-        <v>437</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>471</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="D8" s="8" t="s">
+      <c r="I11" s="12" t="s">
+        <v>449</v>
+      </c>
+      <c r="J11" s="12" t="s">
         <v>439</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>440</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>441</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>442</v>
-      </c>
-      <c r="H8" s="6">
-        <v>3</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>443</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>472</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>438</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>445</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>446</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>447</v>
-      </c>
-      <c r="H9" s="9">
-        <v>4</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>448</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>473</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>405</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>450</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>451</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>452</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>453</v>
-      </c>
-      <c r="H10" s="6">
-        <v>1</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>454</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A11" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>474</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>405</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>455</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>456</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>457</v>
-      </c>
-      <c r="G11" s="13" t="s">
-        <v>458</v>
-      </c>
-      <c r="H11" s="12">
-        <v>2</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>459</v>
-      </c>
-      <c r="J11" s="12" t="s">
-        <v>449</v>
       </c>
     </row>
   </sheetData>
@@ -3996,18 +4017,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0C93C6A-F93F-4793-BD9F-71A4EA325BA6}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.08984375" customWidth="1"/>
-    <col min="3" max="3" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.109375" customWidth="1"/>
+    <col min="3" max="3" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="7" width="40" customWidth="1"/>
-    <col min="8" max="8" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" style="20" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="60" customWidth="1"/>
-    <col min="10" max="10" width="19.08984375" customWidth="1"/>
+    <col min="10" max="10" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4029,7 +4050,7 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="20" t="s">
         <v>7</v>
       </c>
       <c r="I1" t="s">
@@ -4039,324 +4060,324 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="C2" t="s">
+        <v>266</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="H2" s="20">
+        <v>1</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="C3" t="s">
+        <v>274</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E3" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>277</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>278</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="H3" s="20">
+        <v>2</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>279</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="J3" s="5" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>280</v>
       </c>
-      <c r="H2">
+      <c r="C4" t="s">
+        <v>266</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="H4" s="20">
+        <v>3</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="C5" t="s">
+        <v>274</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="H5" s="20">
+        <v>4</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="C6" t="s">
+        <v>274</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="H6" s="20">
         <v>1</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>281</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="C3" t="s">
-        <v>284</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>285</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>286</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>288</v>
-      </c>
-      <c r="H3">
+      <c r="I6" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="C7" t="s">
+        <v>266</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="H7" s="20">
         <v>2</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>289</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>290</v>
-      </c>
-      <c r="C4" t="s">
-        <v>276</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>291</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="H4">
+      <c r="I7" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="C8" t="s">
+        <v>305</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="H8" s="20">
         <v>3</v>
       </c>
-      <c r="I4" s="5" t="s">
-        <v>295</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>296</v>
-      </c>
-      <c r="C5" t="s">
-        <v>284</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>297</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>298</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>300</v>
-      </c>
-      <c r="H5">
+      <c r="I8" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="C9" t="s">
+        <v>305</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="H9" s="20">
         <v>4</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>302</v>
-      </c>
-      <c r="C6" t="s">
-        <v>284</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>303</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>304</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>305</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="H6">
+      <c r="I9" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="C10" t="s">
+        <v>266</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="H10" s="20">
         <v>1</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>307</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="C7" t="s">
-        <v>276</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>310</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="H7">
+      <c r="I10" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="C11" t="s">
+        <v>266</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="H11" s="20">
         <v>2</v>
       </c>
-      <c r="I7" s="5" t="s">
-        <v>313</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="C8" t="s">
-        <v>315</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>316</v>
-      </c>
-      <c r="E8" s="5" t="s">
+      <c r="I11" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="J11" s="5" t="s">
         <v>317</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="H8">
-        <v>3</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="C9" t="s">
-        <v>315</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>322</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>323</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="H9">
-        <v>4</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="C10" t="s">
-        <v>276</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C11" t="s">
-        <v>276</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>337</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>338</v>
-      </c>
-      <c r="H11">
-        <v>2</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>339</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>327</v>
       </c>
     </row>
   </sheetData>
@@ -4370,18 +4391,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C48C580-F830-4656-B607-BD4517683869}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.08984375" customWidth="1"/>
-    <col min="3" max="3" width="22.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.109375" customWidth="1"/>
+    <col min="3" max="3" width="22.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="7" width="40" customWidth="1"/>
-    <col min="8" max="8" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" style="20" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="60" customWidth="1"/>
-    <col min="10" max="10" width="19.08984375" customWidth="1"/>
+    <col min="10" max="10" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4403,7 +4424,7 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="20" t="s">
         <v>7</v>
       </c>
       <c r="I1" t="s">
@@ -4413,324 +4434,324 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>330</v>
+      </c>
+      <c r="C2" t="s">
+        <v>331</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="H2" s="20">
+        <v>1</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="C3" t="s">
+        <v>339</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>340</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E3" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>342</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="H3" s="20">
+        <v>2</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="J3" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="H2">
+      <c r="C4" t="s">
+        <v>331</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>346</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>348</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="H4" s="20">
+        <v>3</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>351</v>
+      </c>
+      <c r="C5" t="s">
+        <v>339</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="H5" s="20">
+        <v>4</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="C6" t="s">
+        <v>339</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="H6" s="20">
         <v>1</v>
       </c>
-      <c r="I2" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>348</v>
-      </c>
-      <c r="C3" t="s">
-        <v>349</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>350</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>351</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>352</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="H3">
+      <c r="I6" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>363</v>
+      </c>
+      <c r="C7" t="s">
+        <v>331</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="H7" s="20">
         <v>2</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>354</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>355</v>
-      </c>
-      <c r="C4" t="s">
-        <v>341</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>359</v>
-      </c>
-      <c r="H4">
+      <c r="I7" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="C8" t="s">
+        <v>370</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>372</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="H8" s="20">
         <v>3</v>
       </c>
-      <c r="I4" s="5" t="s">
-        <v>360</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>361</v>
-      </c>
-      <c r="C5" t="s">
-        <v>349</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>363</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>364</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>365</v>
-      </c>
-      <c r="H5">
+      <c r="I8" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="C9" t="s">
+        <v>370</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="H9" s="20">
         <v>4</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>366</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>367</v>
-      </c>
-      <c r="C6" t="s">
-        <v>349</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>368</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>369</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>371</v>
-      </c>
-      <c r="H6">
+      <c r="I9" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>383</v>
+      </c>
+      <c r="C10" t="s">
+        <v>331</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="H10" s="20">
         <v>1</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>372</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="C7" t="s">
-        <v>341</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>374</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>375</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>376</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>377</v>
-      </c>
-      <c r="H7">
+      <c r="I10" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C11" t="s">
+        <v>331</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>390</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="H11" s="20">
         <v>2</v>
       </c>
-      <c r="I7" s="5" t="s">
-        <v>378</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>379</v>
-      </c>
-      <c r="C8" t="s">
-        <v>380</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>381</v>
-      </c>
-      <c r="E8" s="5" t="s">
+      <c r="I11" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="J11" s="5" t="s">
         <v>382</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>383</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>384</v>
-      </c>
-      <c r="H8">
-        <v>3</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>386</v>
-      </c>
-      <c r="C9" t="s">
-        <v>380</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>387</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>388</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>389</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>390</v>
-      </c>
-      <c r="H9">
-        <v>4</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>391</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>393</v>
-      </c>
-      <c r="C10" t="s">
-        <v>341</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>394</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>395</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>396</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>397</v>
-      </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>398</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>399</v>
-      </c>
-      <c r="C11" t="s">
-        <v>341</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>400</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>401</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>402</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>403</v>
-      </c>
-      <c r="H11">
-        <v>2</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>404</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>392</v>
       </c>
     </row>
   </sheetData>
@@ -4744,18 +4765,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3985FE85-E541-4FD0-B389-FEC482BF15E7}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="49.08984375" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="49.109375" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="7" width="40" customWidth="1"/>
-    <col min="8" max="8" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.21875" style="20" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="60" customWidth="1"/>
-    <col min="10" max="10" width="19.08984375" customWidth="1"/>
+    <col min="10" max="10" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4777,7 +4798,7 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="18" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -4787,324 +4808,324 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="H2" s="2">
+        <v>141</v>
+      </c>
+      <c r="H2" s="19">
         <v>1</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="H3" s="2">
+        <v>148</v>
+      </c>
+      <c r="H3" s="19">
         <v>2</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="H4" s="2">
+        <v>154</v>
+      </c>
+      <c r="H4" s="19">
         <v>3</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="H5" s="2">
+        <v>160</v>
+      </c>
+      <c r="H5" s="19">
         <v>4</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="H6" s="2">
+        <v>166</v>
+      </c>
+      <c r="H6" s="19">
         <v>1</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="H7" s="2">
+        <v>172</v>
+      </c>
+      <c r="H7" s="19">
         <v>2</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="H8" s="2">
+        <v>179</v>
+      </c>
+      <c r="H8" s="19">
         <v>3</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="H9" s="19">
+        <v>4</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="H10" s="19">
+        <v>1</v>
+      </c>
+      <c r="I10" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="J10" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="C11" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="H9" s="2">
-        <v>4</v>
-      </c>
-      <c r="I9" s="2" t="s">
+      <c r="E11" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="F11" s="4" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="2" t="s">
+      <c r="G11" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="H11" s="19">
+        <v>2</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="H10" s="2">
-        <v>1</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="H11" s="2">
-        <v>2</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>209</v>
-      </c>
       <c r="J11" s="2" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -5116,25 +5137,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2aad7df3-4ab7-4daa-980d-cf7206357ce9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101006B71C29808C7F3499BFFC3671560B6FA" ma:contentTypeVersion="8" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="e4f9e1976b194f932bebfa03c600f49f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2aad7df3-4ab7-4daa-980d-cf7206357ce9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8d33a1b74cd678b812bcd025038ca576" ns2:_="">
     <xsd:import namespace="2aad7df3-4ab7-4daa-980d-cf7206357ce9"/>
@@ -5298,25 +5300,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A947F87A-A862-469B-80AB-EC8D5B706ABA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2aad7df3-4ab7-4daa-980d-cf7206357ce9"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79A12AD6-4D28-47C9-A756-6744BC5075CA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2aad7df3-4ab7-4daa-980d-cf7206357ce9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{052D775B-35AE-4D8C-85B8-39FE1C3B4BBC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5332,4 +5335,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79A12AD6-4D28-47C9-A756-6744BC5075CA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A947F87A-A862-469B-80AB-EC8D5B706ABA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2aad7df3-4ab7-4daa-980d-cf7206357ce9"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>